<commit_message>
Sync documentation with demo evolution: per-utility device model + DER assets + combo CA patterns (TDD v1.2, BRFplus v1.2 w/ msg 053 medical dynamic-pricing block, workbook, Runtime v1.1, SDD note, deck URLs/personas); tools canonical for generators
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Enrollment Center/Enrollment Center - BRFplus Configuration Workbook v1.0.xlsx
+++ b/Enrollment Center/Enrollment Center - BRFplus Configuration Workbook v1.0.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>1 (33 messages)</t>
+          <t>1 (34 messages)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1269,7 +1269,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Message Class ZEC_ELIG (33 messages)</t>
+          <t>Message Class ZEC_ELIG (34 messages)</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>055</t>
+          <t>053</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1463,14 +1463,14 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Not compatible with active Prepay service</t>
+          <t>Dynamic peak-event pricing not permitted — Medical Baseline / life-support protection</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>056</t>
+          <t>055</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Prepay and Budget Billing are mutually exclusive</t>
+          <t>Not compatible with active Prepay service</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>057</t>
+          <t>056</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1497,14 +1497,14 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Prepay requires settlement of the active payment plan first</t>
+          <t>Prepay and Budget Billing are mutually exclusive</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>058</t>
+          <t>057</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1514,48 +1514,48 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Only one dynamic rate program allowed — &amp;1 is active</t>
+          <t>Prepay requires settlement of the active payment plan first</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>062</t>
+          <t>058</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Not yet eligible — requires 12 months billing history at premise (&amp;1 of 12)</t>
+          <t>Only one dynamic rate program allowed — &amp;1 is active</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>071</t>
+          <t>062</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>No eligible arrears — program requires a qualifying past-due balance</t>
+          <t>Not yet eligible — requires 12 months billing history at premise (&amp;1 of 12)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>072</t>
+          <t>071</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1565,14 +1565,14 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>No qualifying arrears for a payment plan</t>
+          <t>No eligible arrears — program requires a qualifying past-due balance</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>073</t>
+          <t>072</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1582,14 +1582,14 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>A payment extension is already active until &amp;1</t>
+          <t>No qualifying arrears for a payment plan</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>074</t>
+          <t>073</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Summary billing requires at least two contract accounts</t>
+          <t>A payment extension is already active until &amp;1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>080</t>
+          <t>074</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1616,31 +1616,31 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Curtailable load &amp;1 kW below program minimum &amp;2 kW</t>
+          <t>Summary billing requires at least two contract accounts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>090</t>
+          <t>080</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Not yet eligible — requires an active contract with billing history</t>
+          <t>Curtailable load &amp;1 kW below program minimum &amp;2 kW</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>093</t>
+          <t>090</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1650,31 +1650,31 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Device installation is scheduled after contract activation</t>
+          <t>Not yet eligible — requires an active contract with billing history</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>093</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Vehicle/charger telematics compatibility not yet verified</t>
+          <t>Device installation is scheduled after contract activation</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>320</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1684,14 +1684,14 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Rebate subject to invoice verification</t>
+          <t>Vehicle/charger telematics compatibility not yet verified</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1701,14 +1701,14 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>No valid e-mail address on business partner</t>
+          <t>Rebate subject to invoice verification</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>322</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1718,14 +1718,14 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>&amp;1 defaulted payment plans in last 24 months</t>
+          <t>No valid e-mail address on business partner</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>330</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1735,14 +1735,14 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>&amp;1 payment extensions already granted in last 12 months</t>
+          <t>&amp;1 defaulted payment plans in last 24 months</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>331</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1752,14 +1752,14 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Income verification pending — enrollment provisional</t>
+          <t>&amp;1 payment extensions already granted in last 12 months</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>332</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1769,14 +1769,14 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Physician certification required within 30 days</t>
+          <t>Income verification pending — enrollment provisional</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>333</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1786,14 +1786,14 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Community solar array at capacity — waitlist position assigned</t>
+          <t>Physician certification required within 30 days</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>334</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1803,14 +1803,14 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Interval telemetry certification pending</t>
+          <t>Community solar array at capacity — waitlist position assigned</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>335</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1820,14 +1820,14 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Enrollment replaces the active dynamic rate program &amp;1</t>
+          <t>Interval telemetry certification pending</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>340</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1837,22 +1837,39 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Review stacking with active subscription &amp;1</t>
+          <t>Enrollment replaces the active dynamic rate program &amp;1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
+          <t>341</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Review stacking with active subscription &amp;1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
           <t>342</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>No Wi-Fi at premise — installation survey required</t>
         </is>
@@ -2069,7 +2086,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Generic hard-stop rules read this matrix: each violated criterion appends its fixed message — RATE_CLASS→002/003, AMI→044, AMI_COMM→018, PREPAY block→055/056, MEDICAL→052, BB→056, DPA→012/057, ARREARS→071/072, HISTORY→062(I), LOAD→080, CA_COUNT→074, EXT_ACTIVE→073. PREACTIVE: Y=enrollable at move-in, I=informational only (DT_PREACTIVE_INFO), N=hidden in move-in mode.</t>
+          <t>Generic hard-stop rules read this matrix: each violated criterion appends its fixed message — RATE_CLASS→002/003, AMI→044, AMI_COMM→018, PREPAY block→055/056, MEDICAL→052 (payment) / 053 (dynamic pricing), BB→056, DPA→012/057, ARREARS→071/072, HISTORY→062(I), LOAD→080, CA_COUNT→074, EXT_ACTIVE→073. PREACTIVE: Y=enrollable at move-in, I=informational only (DT_PREACTIVE_INFO), N=hidden in move-in mode.</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2190,11 @@
       </c>
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr"/>
@@ -2251,7 +2272,11 @@
       </c>
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr"/>

</xml_diff>